<commit_message>
Refresh people and computational datasets from source sheets
</commit_message>
<xml_diff>
--- a/inst/extdata/people.xlsx
+++ b/inst/extdata/people.xlsx
@@ -1489,8 +1489,12 @@
       <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="1"/>
-      <c r="F2"/>
+      <c r="E2" s="1" t="n">
+        <v>44228</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2021</v>
+      </c>
       <c r="G2" t="s">
         <v>11</v>
       </c>
@@ -1508,8 +1512,12 @@
       <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="1"/>
-      <c r="F3"/>
+      <c r="E3" s="1" t="n">
+        <v>44458</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2021</v>
+      </c>
       <c r="G3" t="s">
         <v>14</v>
       </c>
@@ -1527,8 +1535,12 @@
       <c r="D4" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4"/>
+      <c r="E4" s="1" t="n">
+        <v>44586</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2022</v>
+      </c>
       <c r="G4" t="s">
         <v>18</v>
       </c>
@@ -1546,8 +1558,12 @@
       <c r="D5" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5"/>
+      <c r="E5" s="1" t="n">
+        <v>44599</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2022</v>
+      </c>
       <c r="G5" t="s">
         <v>21</v>
       </c>
@@ -1565,8 +1581,12 @@
       <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="1"/>
-      <c r="F6"/>
+      <c r="E6" s="1" t="n">
+        <v>44613</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2022</v>
+      </c>
       <c r="G6" t="s">
         <v>23</v>
       </c>
@@ -1584,8 +1604,12 @@
       <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="1"/>
-      <c r="F7"/>
+      <c r="E7" s="1" t="n">
+        <v>44613</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2022</v>
+      </c>
       <c r="G7" t="s">
         <v>25</v>
       </c>
@@ -1603,8 +1627,12 @@
       <c r="D8" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="1"/>
-      <c r="F8"/>
+      <c r="E8" s="1" t="n">
+        <v>44621</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2022</v>
+      </c>
       <c r="G8" t="s">
         <v>27</v>
       </c>
@@ -1622,8 +1650,12 @@
       <c r="D9" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="F9"/>
+      <c r="E9" s="1" t="n">
+        <v>44631</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2022</v>
+      </c>
       <c r="G9" t="s">
         <v>29</v>
       </c>
@@ -1641,8 +1673,12 @@
       <c r="D10" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="1"/>
-      <c r="F10"/>
+      <c r="E10" s="1" t="n">
+        <v>44645</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2022</v>
+      </c>
       <c r="G10" t="s">
         <v>31</v>
       </c>
@@ -1660,8 +1696,12 @@
       <c r="D11" t="s">
         <v>10</v>
       </c>
-      <c r="E11" s="1"/>
-      <c r="F11"/>
+      <c r="E11" s="1" t="n">
+        <v>44652</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2022</v>
+      </c>
       <c r="G11" t="s">
         <v>33</v>
       </c>
@@ -1679,8 +1719,12 @@
       <c r="D12" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="1"/>
-      <c r="F12"/>
+      <c r="E12" s="1" t="n">
+        <v>44655</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2022</v>
+      </c>
       <c r="G12" t="s">
         <v>35</v>
       </c>
@@ -1698,8 +1742,12 @@
       <c r="D13" t="s">
         <v>10</v>
       </c>
-      <c r="E13" s="1"/>
-      <c r="F13"/>
+      <c r="E13" s="1" t="n">
+        <v>44682</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2022</v>
+      </c>
       <c r="G13" t="s">
         <v>37</v>
       </c>
@@ -1717,8 +1765,12 @@
       <c r="D14" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="1"/>
-      <c r="F14"/>
+      <c r="E14" s="1" t="n">
+        <v>44682</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2022</v>
+      </c>
       <c r="G14" t="s">
         <v>39</v>
       </c>
@@ -1736,8 +1788,12 @@
       <c r="D15" t="s">
         <v>10</v>
       </c>
-      <c r="E15" s="1"/>
-      <c r="F15"/>
+      <c r="E15" s="1" t="n">
+        <v>44713</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2022</v>
+      </c>
       <c r="G15" t="s">
         <v>41</v>
       </c>
@@ -1755,8 +1811,12 @@
       <c r="D16" t="s">
         <v>10</v>
       </c>
-      <c r="E16" s="1"/>
-      <c r="F16"/>
+      <c r="E16" s="1" t="n">
+        <v>44725</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2022</v>
+      </c>
       <c r="G16" t="s">
         <v>43</v>
       </c>
@@ -1774,8 +1834,12 @@
       <c r="D17" t="s">
         <v>10</v>
       </c>
-      <c r="E17" s="1"/>
-      <c r="F17"/>
+      <c r="E17" s="1" t="n">
+        <v>44774</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2022</v>
+      </c>
       <c r="G17" t="s">
         <v>45</v>
       </c>
@@ -1793,8 +1857,12 @@
       <c r="D18" t="s">
         <v>10</v>
       </c>
-      <c r="E18" s="1"/>
-      <c r="F18"/>
+      <c r="E18" s="1" t="n">
+        <v>44774</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2022</v>
+      </c>
       <c r="G18" t="s">
         <v>47</v>
       </c>
@@ -1812,8 +1880,12 @@
       <c r="D19" t="s">
         <v>10</v>
       </c>
-      <c r="E19" s="1"/>
-      <c r="F19"/>
+      <c r="E19" s="1" t="n">
+        <v>44805</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2022</v>
+      </c>
       <c r="G19" t="s">
         <v>49</v>
       </c>
@@ -1831,8 +1903,12 @@
       <c r="D20" t="s">
         <v>10</v>
       </c>
-      <c r="E20" s="1"/>
-      <c r="F20"/>
+      <c r="E20" s="1" t="n">
+        <v>44805</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2022</v>
+      </c>
       <c r="G20" t="s">
         <v>51</v>
       </c>
@@ -1850,8 +1926,12 @@
       <c r="D21" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="1"/>
-      <c r="F21"/>
+      <c r="E21" s="1" t="n">
+        <v>44820</v>
+      </c>
+      <c r="F21" t="n">
+        <v>2022</v>
+      </c>
       <c r="G21" t="s">
         <v>53</v>
       </c>
@@ -1869,8 +1949,12 @@
       <c r="D22" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="1"/>
-      <c r="F22"/>
+      <c r="E22" s="1" t="n">
+        <v>44820</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2022</v>
+      </c>
       <c r="G22" t="s">
         <v>55</v>
       </c>
@@ -1888,8 +1972,12 @@
       <c r="D23" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="1"/>
-      <c r="F23"/>
+      <c r="E23" s="1" t="n">
+        <v>44820</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2022</v>
+      </c>
       <c r="G23" t="s">
         <v>57</v>
       </c>
@@ -1907,8 +1995,12 @@
       <c r="D24" t="s">
         <v>10</v>
       </c>
-      <c r="E24" s="1"/>
-      <c r="F24"/>
+      <c r="E24" s="1" t="n">
+        <v>44835</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2022</v>
+      </c>
       <c r="G24" t="s">
         <v>59</v>
       </c>
@@ -1926,8 +2018,12 @@
       <c r="D25" t="s">
         <v>10</v>
       </c>
-      <c r="E25" s="1"/>
-      <c r="F25"/>
+      <c r="E25" s="1" t="n">
+        <v>44835</v>
+      </c>
+      <c r="F25" t="n">
+        <v>2022</v>
+      </c>
       <c r="G25" t="s">
         <v>61</v>
       </c>
@@ -1945,8 +2041,12 @@
       <c r="D26" t="s">
         <v>10</v>
       </c>
-      <c r="E26" s="1"/>
-      <c r="F26"/>
+      <c r="E26" s="1" t="n">
+        <v>44835</v>
+      </c>
+      <c r="F26" t="n">
+        <v>2022</v>
+      </c>
       <c r="G26" t="s">
         <v>63</v>
       </c>
@@ -1964,8 +2064,12 @@
       <c r="D27" t="s">
         <v>10</v>
       </c>
-      <c r="E27" s="1"/>
-      <c r="F27"/>
+      <c r="E27" s="1" t="n">
+        <v>44881</v>
+      </c>
+      <c r="F27" t="n">
+        <v>2022</v>
+      </c>
       <c r="G27" t="s">
         <v>65</v>
       </c>
@@ -1983,8 +2087,12 @@
       <c r="D28" t="s">
         <v>17</v>
       </c>
-      <c r="E28" s="1"/>
-      <c r="F28"/>
+      <c r="E28" s="1" t="n">
+        <v>44927</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2023</v>
+      </c>
       <c r="G28" t="s">
         <v>69</v>
       </c>
@@ -2002,8 +2110,12 @@
       <c r="D29" t="s">
         <v>10</v>
       </c>
-      <c r="E29" s="1"/>
-      <c r="F29"/>
+      <c r="E29" s="1" t="n">
+        <v>44930</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2023</v>
+      </c>
       <c r="G29" t="s">
         <v>71</v>
       </c>
@@ -2021,8 +2133,12 @@
       <c r="D30" t="s">
         <v>10</v>
       </c>
-      <c r="E30" s="1"/>
-      <c r="F30"/>
+      <c r="E30" s="1" t="n">
+        <v>44958</v>
+      </c>
+      <c r="F30" t="n">
+        <v>2023</v>
+      </c>
       <c r="G30" t="s">
         <v>73</v>
       </c>
@@ -2040,8 +2156,12 @@
       <c r="D31" t="s">
         <v>10</v>
       </c>
-      <c r="E31" s="1"/>
-      <c r="F31"/>
+      <c r="E31" s="1" t="n">
+        <v>44977</v>
+      </c>
+      <c r="F31" t="n">
+        <v>2023</v>
+      </c>
       <c r="G31" t="s">
         <v>75</v>
       </c>
@@ -2059,8 +2179,12 @@
       <c r="D32" t="s">
         <v>10</v>
       </c>
-      <c r="E32" s="1"/>
-      <c r="F32"/>
+      <c r="E32" s="1" t="n">
+        <v>44986</v>
+      </c>
+      <c r="F32" t="n">
+        <v>2023</v>
+      </c>
       <c r="G32" t="s">
         <v>77</v>
       </c>
@@ -2078,8 +2202,12 @@
       <c r="D33" t="s">
         <v>10</v>
       </c>
-      <c r="E33" s="1"/>
-      <c r="F33"/>
+      <c r="E33" s="1" t="n">
+        <v>44986</v>
+      </c>
+      <c r="F33" t="n">
+        <v>2023</v>
+      </c>
       <c r="G33" t="s">
         <v>79</v>
       </c>
@@ -2097,8 +2225,12 @@
       <c r="D34" t="s">
         <v>10</v>
       </c>
-      <c r="E34" s="1"/>
-      <c r="F34"/>
+      <c r="E34" s="1" t="n">
+        <v>44986</v>
+      </c>
+      <c r="F34" t="n">
+        <v>2023</v>
+      </c>
       <c r="G34" t="s">
         <v>81</v>
       </c>
@@ -2116,8 +2248,12 @@
       <c r="D35" t="s">
         <v>10</v>
       </c>
-      <c r="E35" s="1"/>
-      <c r="F35"/>
+      <c r="E35" s="1" t="n">
+        <v>45001</v>
+      </c>
+      <c r="F35" t="n">
+        <v>2023</v>
+      </c>
       <c r="G35" t="s">
         <v>83</v>
       </c>
@@ -2135,8 +2271,12 @@
       <c r="D36" t="s">
         <v>10</v>
       </c>
-      <c r="E36" s="1"/>
-      <c r="F36"/>
+      <c r="E36" s="1" t="n">
+        <v>45038</v>
+      </c>
+      <c r="F36" t="n">
+        <v>2023</v>
+      </c>
       <c r="G36" t="s">
         <v>85</v>
       </c>
@@ -2154,8 +2294,12 @@
       <c r="D37" t="s">
         <v>17</v>
       </c>
-      <c r="E37" s="1"/>
-      <c r="F37"/>
+      <c r="E37" s="1" t="n">
+        <v>45047</v>
+      </c>
+      <c r="F37" t="n">
+        <v>2023</v>
+      </c>
       <c r="G37"/>
     </row>
     <row r="38">
@@ -2171,8 +2315,12 @@
       <c r="D38" t="s">
         <v>10</v>
       </c>
-      <c r="E38" s="1"/>
-      <c r="F38"/>
+      <c r="E38" s="1" t="n">
+        <v>45055</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2023</v>
+      </c>
       <c r="G38" t="s">
         <v>89</v>
       </c>
@@ -2190,8 +2338,12 @@
       <c r="D39" t="s">
         <v>17</v>
       </c>
-      <c r="E39" s="1"/>
-      <c r="F39"/>
+      <c r="E39" s="1" t="n">
+        <v>45061</v>
+      </c>
+      <c r="F39" t="n">
+        <v>2023</v>
+      </c>
       <c r="G39"/>
     </row>
     <row r="40">
@@ -2207,8 +2359,12 @@
       <c r="D40" t="s">
         <v>10</v>
       </c>
-      <c r="E40" s="1"/>
-      <c r="F40"/>
+      <c r="E40" s="1" t="n">
+        <v>45187</v>
+      </c>
+      <c r="F40" t="n">
+        <v>2023</v>
+      </c>
       <c r="G40" t="s">
         <v>92</v>
       </c>
@@ -2226,8 +2382,12 @@
       <c r="D41" t="s">
         <v>10</v>
       </c>
-      <c r="E41" s="1"/>
-      <c r="F41"/>
+      <c r="E41" s="1" t="n">
+        <v>45187</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2023</v>
+      </c>
       <c r="G41" t="s">
         <v>94</v>
       </c>
@@ -2245,8 +2405,12 @@
       <c r="D42" t="s">
         <v>10</v>
       </c>
-      <c r="E42" s="1"/>
-      <c r="F42"/>
+      <c r="E42" s="1" t="n">
+        <v>45187</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2023</v>
+      </c>
       <c r="G42" t="s">
         <v>96</v>
       </c>
@@ -2264,8 +2428,12 @@
       <c r="D43" t="s">
         <v>10</v>
       </c>
-      <c r="E43" s="1"/>
-      <c r="F43"/>
+      <c r="E43" s="1" t="n">
+        <v>45187</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2023</v>
+      </c>
       <c r="G43" t="s">
         <v>98</v>
       </c>
@@ -2283,8 +2451,12 @@
       <c r="D44" t="s">
         <v>10</v>
       </c>
-      <c r="E44" s="1"/>
-      <c r="F44"/>
+      <c r="E44" s="1" t="n">
+        <v>45187</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2023</v>
+      </c>
       <c r="G44" t="s">
         <v>100</v>
       </c>
@@ -2302,8 +2474,12 @@
       <c r="D45" t="s">
         <v>10</v>
       </c>
-      <c r="E45" s="1"/>
-      <c r="F45"/>
+      <c r="E45" s="1" t="n">
+        <v>45194</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2023</v>
+      </c>
       <c r="G45" t="s">
         <v>102</v>
       </c>
@@ -2321,8 +2497,12 @@
       <c r="D46" t="s">
         <v>10</v>
       </c>
-      <c r="E46" s="1"/>
-      <c r="F46"/>
+      <c r="E46" s="1" t="n">
+        <v>45200</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2023</v>
+      </c>
       <c r="G46" t="s">
         <v>104</v>
       </c>
@@ -2340,8 +2520,12 @@
       <c r="D47" t="s">
         <v>10</v>
       </c>
-      <c r="E47" s="1"/>
-      <c r="F47"/>
+      <c r="E47" s="1" t="n">
+        <v>45200</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2023</v>
+      </c>
       <c r="G47" t="s">
         <v>106</v>
       </c>
@@ -2359,8 +2543,12 @@
       <c r="D48" t="s">
         <v>17</v>
       </c>
-      <c r="E48" s="1"/>
-      <c r="F48"/>
+      <c r="E48" s="1" t="n">
+        <v>45200</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2023</v>
+      </c>
       <c r="G48"/>
     </row>
     <row r="49">
@@ -2376,8 +2564,12 @@
       <c r="D49" t="s">
         <v>10</v>
       </c>
-      <c r="E49" s="1"/>
-      <c r="F49"/>
+      <c r="E49" s="1" t="n">
+        <v>45201</v>
+      </c>
+      <c r="F49" t="n">
+        <v>2023</v>
+      </c>
       <c r="G49" t="s">
         <v>110</v>
       </c>
@@ -2395,8 +2587,12 @@
       <c r="D50" t="s">
         <v>10</v>
       </c>
-      <c r="E50" s="1"/>
-      <c r="F50"/>
+      <c r="E50" s="1" t="n">
+        <v>45201</v>
+      </c>
+      <c r="F50" t="n">
+        <v>2023</v>
+      </c>
       <c r="G50" t="s">
         <v>112</v>
       </c>
@@ -2414,8 +2610,12 @@
       <c r="D51" t="s">
         <v>10</v>
       </c>
-      <c r="E51" s="1"/>
-      <c r="F51"/>
+      <c r="E51" s="1" t="n">
+        <v>45201</v>
+      </c>
+      <c r="F51" t="n">
+        <v>2023</v>
+      </c>
       <c r="G51" t="s">
         <v>114</v>
       </c>
@@ -2433,8 +2633,12 @@
       <c r="D52" t="s">
         <v>10</v>
       </c>
-      <c r="E52" s="1"/>
-      <c r="F52"/>
+      <c r="E52" s="1" t="n">
+        <v>45201</v>
+      </c>
+      <c r="F52" t="n">
+        <v>2023</v>
+      </c>
       <c r="G52" t="s">
         <v>116</v>
       </c>
@@ -2452,8 +2656,12 @@
       <c r="D53" t="s">
         <v>10</v>
       </c>
-      <c r="E53" s="1"/>
-      <c r="F53"/>
+      <c r="E53" s="1" t="n">
+        <v>45209</v>
+      </c>
+      <c r="F53" t="n">
+        <v>2023</v>
+      </c>
       <c r="G53" t="s">
         <v>118</v>
       </c>
@@ -2471,8 +2679,12 @@
       <c r="D54" t="s">
         <v>17</v>
       </c>
-      <c r="E54" s="1"/>
-      <c r="F54"/>
+      <c r="E54" s="1" t="n">
+        <v>45216</v>
+      </c>
+      <c r="F54" t="n">
+        <v>2023</v>
+      </c>
       <c r="G54"/>
     </row>
     <row r="55">
@@ -2488,8 +2700,12 @@
       <c r="D55" t="s">
         <v>17</v>
       </c>
-      <c r="E55" s="1"/>
-      <c r="F55"/>
+      <c r="E55" s="1" t="n">
+        <v>45306</v>
+      </c>
+      <c r="F55" t="n">
+        <v>2024</v>
+      </c>
       <c r="G55"/>
     </row>
     <row r="56">
@@ -2505,8 +2721,12 @@
       <c r="D56" t="s">
         <v>10</v>
       </c>
-      <c r="E56" s="1"/>
-      <c r="F56"/>
+      <c r="E56" s="1" t="n">
+        <v>45334</v>
+      </c>
+      <c r="F56" t="n">
+        <v>2024</v>
+      </c>
       <c r="G56" t="s">
         <v>122</v>
       </c>
@@ -2524,8 +2744,12 @@
       <c r="D57" t="s">
         <v>10</v>
       </c>
-      <c r="E57" s="1"/>
-      <c r="F57"/>
+      <c r="E57" s="1" t="n">
+        <v>45341</v>
+      </c>
+      <c r="F57" t="n">
+        <v>2024</v>
+      </c>
       <c r="G57" t="s">
         <v>124</v>
       </c>
@@ -2543,8 +2767,12 @@
       <c r="D58" t="s">
         <v>10</v>
       </c>
-      <c r="E58" s="1"/>
-      <c r="F58"/>
+      <c r="E58" s="1" t="n">
+        <v>45348</v>
+      </c>
+      <c r="F58" t="n">
+        <v>2024</v>
+      </c>
       <c r="G58" t="s">
         <v>126</v>
       </c>
@@ -2560,8 +2788,12 @@
       <c r="D59" t="s">
         <v>10</v>
       </c>
-      <c r="E59" s="1"/>
-      <c r="F59"/>
+      <c r="E59" s="1" t="n">
+        <v>45348</v>
+      </c>
+      <c r="F59" t="n">
+        <v>2024</v>
+      </c>
       <c r="G59" t="s">
         <v>127</v>
       </c>
@@ -2579,8 +2811,12 @@
       <c r="D60" t="s">
         <v>10</v>
       </c>
-      <c r="E60" s="1"/>
-      <c r="F60"/>
+      <c r="E60" s="1" t="n">
+        <v>45349</v>
+      </c>
+      <c r="F60" t="n">
+        <v>2024</v>
+      </c>
       <c r="G60" t="s">
         <v>129</v>
       </c>
@@ -2598,8 +2834,12 @@
       <c r="D61" t="s">
         <v>10</v>
       </c>
-      <c r="E61" s="1"/>
-      <c r="F61"/>
+      <c r="E61" s="1" t="n">
+        <v>45352</v>
+      </c>
+      <c r="F61" t="n">
+        <v>2024</v>
+      </c>
       <c r="G61" t="s">
         <v>131</v>
       </c>
@@ -2617,8 +2857,12 @@
       <c r="D62" t="s">
         <v>17</v>
       </c>
-      <c r="E62" s="1"/>
-      <c r="F62"/>
+      <c r="E62" s="1" t="n">
+        <v>45352</v>
+      </c>
+      <c r="F62" t="n">
+        <v>2024</v>
+      </c>
       <c r="G62"/>
     </row>
     <row r="63">
@@ -2634,8 +2878,12 @@
       <c r="D63" t="s">
         <v>10</v>
       </c>
-      <c r="E63" s="1"/>
-      <c r="F63"/>
+      <c r="E63" s="1" t="n">
+        <v>45355</v>
+      </c>
+      <c r="F63" t="n">
+        <v>2024</v>
+      </c>
       <c r="G63" t="s">
         <v>134</v>
       </c>
@@ -2653,8 +2901,12 @@
       <c r="D64" t="s">
         <v>10</v>
       </c>
-      <c r="E64" s="1"/>
-      <c r="F64"/>
+      <c r="E64" s="1" t="n">
+        <v>45355</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2024</v>
+      </c>
       <c r="G64" t="s">
         <v>136</v>
       </c>
@@ -2672,8 +2924,12 @@
       <c r="D65" t="s">
         <v>10</v>
       </c>
-      <c r="E65" s="1"/>
-      <c r="F65"/>
+      <c r="E65" s="1" t="n">
+        <v>45355</v>
+      </c>
+      <c r="F65" t="n">
+        <v>2024</v>
+      </c>
       <c r="G65" t="s">
         <v>138</v>
       </c>
@@ -2691,8 +2947,12 @@
       <c r="D66" t="s">
         <v>10</v>
       </c>
-      <c r="E66" s="1"/>
-      <c r="F66"/>
+      <c r="E66" s="1" t="n">
+        <v>45355</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2024</v>
+      </c>
       <c r="G66" t="s">
         <v>140</v>
       </c>
@@ -2710,8 +2970,12 @@
       <c r="D67" t="s">
         <v>10</v>
       </c>
-      <c r="E67" s="1"/>
-      <c r="F67"/>
+      <c r="E67" s="1" t="n">
+        <v>45355</v>
+      </c>
+      <c r="F67" t="n">
+        <v>2024</v>
+      </c>
       <c r="G67" t="s">
         <v>142</v>
       </c>
@@ -2729,8 +2993,12 @@
       <c r="D68" t="s">
         <v>10</v>
       </c>
-      <c r="E68" s="1"/>
-      <c r="F68"/>
+      <c r="E68" s="1" t="n">
+        <v>45355</v>
+      </c>
+      <c r="F68" t="n">
+        <v>2024</v>
+      </c>
       <c r="G68" t="s">
         <v>144</v>
       </c>
@@ -2748,8 +3016,12 @@
       <c r="D69" t="s">
         <v>10</v>
       </c>
-      <c r="E69" s="1"/>
-      <c r="F69"/>
+      <c r="E69" s="1" t="n">
+        <v>45362</v>
+      </c>
+      <c r="F69" t="n">
+        <v>2024</v>
+      </c>
       <c r="G69" t="s">
         <v>146</v>
       </c>
@@ -2767,8 +3039,12 @@
       <c r="D70" t="s">
         <v>10</v>
       </c>
-      <c r="E70" s="1"/>
-      <c r="F70"/>
+      <c r="E70" s="1" t="n">
+        <v>45362</v>
+      </c>
+      <c r="F70" t="n">
+        <v>2024</v>
+      </c>
       <c r="G70" t="s">
         <v>148</v>
       </c>
@@ -2786,8 +3062,12 @@
       <c r="D71" t="s">
         <v>10</v>
       </c>
-      <c r="E71" s="1"/>
-      <c r="F71"/>
+      <c r="E71" s="1" t="n">
+        <v>45366</v>
+      </c>
+      <c r="F71" t="n">
+        <v>2024</v>
+      </c>
       <c r="G71" t="s">
         <v>150</v>
       </c>
@@ -2805,8 +3085,12 @@
       <c r="D72" t="s">
         <v>10</v>
       </c>
-      <c r="E72" s="1"/>
-      <c r="F72"/>
+      <c r="E72" s="1" t="n">
+        <v>45369</v>
+      </c>
+      <c r="F72" t="n">
+        <v>2024</v>
+      </c>
       <c r="G72" t="s">
         <v>152</v>
       </c>
@@ -2824,8 +3108,12 @@
       <c r="D73" t="s">
         <v>10</v>
       </c>
-      <c r="E73" s="1"/>
-      <c r="F73"/>
+      <c r="E73" s="1" t="n">
+        <v>45383</v>
+      </c>
+      <c r="F73" t="n">
+        <v>2024</v>
+      </c>
       <c r="G73" t="s">
         <v>154</v>
       </c>
@@ -2843,8 +3131,12 @@
       <c r="D74" t="s">
         <v>10</v>
       </c>
-      <c r="E74" s="1"/>
-      <c r="F74"/>
+      <c r="E74" s="1" t="n">
+        <v>45383</v>
+      </c>
+      <c r="F74" t="n">
+        <v>2024</v>
+      </c>
       <c r="G74" t="s">
         <v>156</v>
       </c>
@@ -2862,8 +3154,12 @@
       <c r="D75" t="s">
         <v>10</v>
       </c>
-      <c r="E75" s="1"/>
-      <c r="F75"/>
+      <c r="E75" s="1" t="n">
+        <v>45391</v>
+      </c>
+      <c r="F75" t="n">
+        <v>2024</v>
+      </c>
       <c r="G75" t="s">
         <v>158</v>
       </c>
@@ -2881,8 +3177,12 @@
       <c r="D76" t="s">
         <v>17</v>
       </c>
-      <c r="E76" s="1"/>
-      <c r="F76"/>
+      <c r="E76" s="1" t="n">
+        <v>45474</v>
+      </c>
+      <c r="F76" t="n">
+        <v>2024</v>
+      </c>
       <c r="G76" t="s">
         <v>160</v>
       </c>
@@ -2900,8 +3200,12 @@
       <c r="D77" t="s">
         <v>17</v>
       </c>
-      <c r="E77" s="1"/>
-      <c r="F77"/>
+      <c r="E77" s="1" t="n">
+        <v>45474</v>
+      </c>
+      <c r="F77" t="n">
+        <v>2024</v>
+      </c>
       <c r="G77"/>
     </row>
     <row r="78">
@@ -2917,8 +3221,12 @@
       <c r="D78" t="s">
         <v>17</v>
       </c>
-      <c r="E78" s="1"/>
-      <c r="F78"/>
+      <c r="E78" s="1" t="n">
+        <v>45488</v>
+      </c>
+      <c r="F78" t="n">
+        <v>2024</v>
+      </c>
       <c r="G78"/>
     </row>
     <row r="79">
@@ -2934,8 +3242,12 @@
       <c r="D79" t="s">
         <v>17</v>
       </c>
-      <c r="E79" s="1"/>
-      <c r="F79"/>
+      <c r="E79" s="1" t="n">
+        <v>45495</v>
+      </c>
+      <c r="F79" t="n">
+        <v>2024</v>
+      </c>
       <c r="G79"/>
     </row>
     <row r="80">
@@ -2951,8 +3263,12 @@
       <c r="D80" t="s">
         <v>10</v>
       </c>
-      <c r="E80" s="1"/>
-      <c r="F80"/>
+      <c r="E80" s="1" t="n">
+        <v>45502</v>
+      </c>
+      <c r="F80" t="n">
+        <v>2024</v>
+      </c>
       <c r="G80" t="s">
         <v>166</v>
       </c>
@@ -2970,8 +3286,12 @@
       <c r="D81" t="s">
         <v>10</v>
       </c>
-      <c r="E81" s="1"/>
-      <c r="F81"/>
+      <c r="E81" s="1" t="n">
+        <v>45523</v>
+      </c>
+      <c r="F81" t="n">
+        <v>2024</v>
+      </c>
       <c r="G81" t="s">
         <v>168</v>
       </c>
@@ -2989,8 +3309,12 @@
       <c r="D82" t="s">
         <v>10</v>
       </c>
-      <c r="E82" s="1"/>
-      <c r="F82"/>
+      <c r="E82" s="1" t="n">
+        <v>45549</v>
+      </c>
+      <c r="F82" t="n">
+        <v>2024</v>
+      </c>
       <c r="G82" t="s">
         <v>170</v>
       </c>
@@ -3008,8 +3332,12 @@
       <c r="D83" t="s">
         <v>10</v>
       </c>
-      <c r="E83" s="1"/>
-      <c r="F83"/>
+      <c r="E83" s="1" t="n">
+        <v>45551</v>
+      </c>
+      <c r="F83" t="n">
+        <v>2024</v>
+      </c>
       <c r="G83" t="s">
         <v>172</v>
       </c>
@@ -3027,8 +3355,12 @@
       <c r="D84" t="s">
         <v>10</v>
       </c>
-      <c r="E84" s="1"/>
-      <c r="F84"/>
+      <c r="E84" s="1" t="n">
+        <v>45551</v>
+      </c>
+      <c r="F84" t="n">
+        <v>2024</v>
+      </c>
       <c r="G84" t="s">
         <v>174</v>
       </c>
@@ -3046,8 +3378,12 @@
       <c r="D85" t="s">
         <v>10</v>
       </c>
-      <c r="E85" s="1"/>
-      <c r="F85"/>
+      <c r="E85" s="1" t="n">
+        <v>45551</v>
+      </c>
+      <c r="F85" t="n">
+        <v>2024</v>
+      </c>
       <c r="G85" t="s">
         <v>176</v>
       </c>
@@ -3065,8 +3401,12 @@
       <c r="D86" t="s">
         <v>10</v>
       </c>
-      <c r="E86" s="1"/>
-      <c r="F86"/>
+      <c r="E86" s="1" t="n">
+        <v>45557</v>
+      </c>
+      <c r="F86" t="n">
+        <v>2024</v>
+      </c>
       <c r="G86" t="s">
         <v>178</v>
       </c>
@@ -3084,8 +3424,12 @@
       <c r="D87" t="s">
         <v>10</v>
       </c>
-      <c r="E87" s="1"/>
-      <c r="F87"/>
+      <c r="E87" s="1" t="n">
+        <v>45558</v>
+      </c>
+      <c r="F87" t="n">
+        <v>2024</v>
+      </c>
       <c r="G87" t="s">
         <v>180</v>
       </c>
@@ -3103,8 +3447,12 @@
       <c r="D88" t="s">
         <v>10</v>
       </c>
-      <c r="E88" s="1"/>
-      <c r="F88"/>
+      <c r="E88" s="1" t="n">
+        <v>45558</v>
+      </c>
+      <c r="F88" t="n">
+        <v>2024</v>
+      </c>
       <c r="G88" t="s">
         <v>182</v>
       </c>
@@ -3122,8 +3470,12 @@
       <c r="D89" t="s">
         <v>10</v>
       </c>
-      <c r="E89" s="1"/>
-      <c r="F89"/>
+      <c r="E89" s="1" t="n">
+        <v>45558</v>
+      </c>
+      <c r="F89" t="n">
+        <v>2024</v>
+      </c>
       <c r="G89" t="s">
         <v>184</v>
       </c>
@@ -3141,8 +3493,12 @@
       <c r="D90" t="s">
         <v>10</v>
       </c>
-      <c r="E90" s="1"/>
-      <c r="F90"/>
+      <c r="E90" s="1" t="n">
+        <v>45565</v>
+      </c>
+      <c r="F90" t="n">
+        <v>2024</v>
+      </c>
       <c r="G90" t="s">
         <v>186</v>
       </c>
@@ -3160,8 +3516,12 @@
       <c r="D91" t="s">
         <v>10</v>
       </c>
-      <c r="E91" s="1"/>
-      <c r="F91"/>
+      <c r="E91" s="1" t="n">
+        <v>45566</v>
+      </c>
+      <c r="F91" t="n">
+        <v>2024</v>
+      </c>
       <c r="G91" t="s">
         <v>188</v>
       </c>
@@ -3179,8 +3539,12 @@
       <c r="D92" t="s">
         <v>10</v>
       </c>
-      <c r="E92" s="1"/>
-      <c r="F92"/>
+      <c r="E92" s="1" t="n">
+        <v>45566</v>
+      </c>
+      <c r="F92" t="n">
+        <v>2024</v>
+      </c>
       <c r="G92" t="s">
         <v>190</v>
       </c>
@@ -3198,8 +3562,12 @@
       <c r="D93" t="s">
         <v>10</v>
       </c>
-      <c r="E93" s="1"/>
-      <c r="F93"/>
+      <c r="E93" s="1" t="n">
+        <v>45566</v>
+      </c>
+      <c r="F93" t="n">
+        <v>2024</v>
+      </c>
       <c r="G93" t="s">
         <v>192</v>
       </c>
@@ -3217,8 +3585,12 @@
       <c r="D94" t="s">
         <v>10</v>
       </c>
-      <c r="E94" s="1"/>
-      <c r="F94"/>
+      <c r="E94" s="1" t="n">
+        <v>45566</v>
+      </c>
+      <c r="F94" t="n">
+        <v>2024</v>
+      </c>
       <c r="G94" t="s">
         <v>194</v>
       </c>
@@ -3236,8 +3608,12 @@
       <c r="D95" t="s">
         <v>10</v>
       </c>
-      <c r="E95" s="1"/>
-      <c r="F95"/>
+      <c r="E95" s="1" t="n">
+        <v>45569</v>
+      </c>
+      <c r="F95" t="n">
+        <v>2024</v>
+      </c>
       <c r="G95" t="s">
         <v>196</v>
       </c>
@@ -3255,8 +3631,12 @@
       <c r="D96" t="s">
         <v>10</v>
       </c>
-      <c r="E96" s="1"/>
-      <c r="F96"/>
+      <c r="E96" s="1" t="n">
+        <v>45586</v>
+      </c>
+      <c r="F96" t="n">
+        <v>2024</v>
+      </c>
       <c r="G96" t="s">
         <v>198</v>
       </c>
@@ -3274,8 +3654,12 @@
       <c r="D97" t="s">
         <v>10</v>
       </c>
-      <c r="E97" s="1"/>
-      <c r="F97"/>
+      <c r="E97" s="1" t="n">
+        <v>45587</v>
+      </c>
+      <c r="F97" t="n">
+        <v>2024</v>
+      </c>
       <c r="G97" t="s">
         <v>200</v>
       </c>
@@ -3293,8 +3677,12 @@
       <c r="D98" t="s">
         <v>17</v>
       </c>
-      <c r="E98" s="1"/>
-      <c r="F98"/>
+      <c r="E98" s="1" t="n">
+        <v>45597</v>
+      </c>
+      <c r="F98" t="n">
+        <v>2024</v>
+      </c>
       <c r="G98"/>
     </row>
     <row r="99">
@@ -3310,8 +3698,12 @@
       <c r="D99" t="s">
         <v>10</v>
       </c>
-      <c r="E99" s="1"/>
-      <c r="F99"/>
+      <c r="E99" s="1" t="n">
+        <v>45667</v>
+      </c>
+      <c r="F99" t="n">
+        <v>2025</v>
+      </c>
       <c r="G99" t="s">
         <v>204</v>
       </c>
@@ -3329,8 +3721,12 @@
       <c r="D100" t="s">
         <v>10</v>
       </c>
-      <c r="E100" s="1"/>
-      <c r="F100"/>
+      <c r="E100" s="1" t="n">
+        <v>45672</v>
+      </c>
+      <c r="F100" t="n">
+        <v>2025</v>
+      </c>
       <c r="G100" t="s">
         <v>206</v>
       </c>
@@ -3348,8 +3744,12 @@
       <c r="D101" t="s">
         <v>10</v>
       </c>
-      <c r="E101" s="1"/>
-      <c r="F101"/>
+      <c r="E101" s="1" t="n">
+        <v>45698</v>
+      </c>
+      <c r="F101" t="n">
+        <v>2025</v>
+      </c>
       <c r="G101" t="s">
         <v>208</v>
       </c>
@@ -3367,8 +3767,12 @@
       <c r="D102" t="s">
         <v>10</v>
       </c>
-      <c r="E102" s="1"/>
-      <c r="F102"/>
+      <c r="E102" s="1" t="n">
+        <v>45698</v>
+      </c>
+      <c r="F102" t="n">
+        <v>2025</v>
+      </c>
       <c r="G102" t="s">
         <v>210</v>
       </c>
@@ -3386,8 +3790,12 @@
       <c r="D103" t="s">
         <v>10</v>
       </c>
-      <c r="E103" s="1"/>
-      <c r="F103"/>
+      <c r="E103" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F103" t="n">
+        <v>2025</v>
+      </c>
       <c r="G103" t="s">
         <v>212</v>
       </c>
@@ -3405,8 +3813,12 @@
       <c r="D104" t="s">
         <v>10</v>
       </c>
-      <c r="E104" s="1"/>
-      <c r="F104"/>
+      <c r="E104" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F104" t="n">
+        <v>2025</v>
+      </c>
       <c r="G104" t="s">
         <v>214</v>
       </c>
@@ -3424,8 +3836,12 @@
       <c r="D105" t="s">
         <v>10</v>
       </c>
-      <c r="E105" s="1"/>
-      <c r="F105"/>
+      <c r="E105" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F105" t="n">
+        <v>2025</v>
+      </c>
       <c r="G105" t="s">
         <v>216</v>
       </c>
@@ -3443,8 +3859,12 @@
       <c r="D106" t="s">
         <v>10</v>
       </c>
-      <c r="E106" s="1"/>
-      <c r="F106"/>
+      <c r="E106" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F106" t="n">
+        <v>2025</v>
+      </c>
       <c r="G106" t="s">
         <v>218</v>
       </c>
@@ -3462,8 +3882,12 @@
       <c r="D107" t="s">
         <v>10</v>
       </c>
-      <c r="E107" s="1"/>
-      <c r="F107"/>
+      <c r="E107" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F107" t="n">
+        <v>2025</v>
+      </c>
       <c r="G107" t="s">
         <v>220</v>
       </c>
@@ -3481,8 +3905,12 @@
       <c r="D108" t="s">
         <v>10</v>
       </c>
-      <c r="E108" s="1"/>
-      <c r="F108"/>
+      <c r="E108" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F108" t="n">
+        <v>2025</v>
+      </c>
       <c r="G108" t="s">
         <v>222</v>
       </c>
@@ -3500,8 +3928,12 @@
       <c r="D109" t="s">
         <v>10</v>
       </c>
-      <c r="E109" s="1"/>
-      <c r="F109"/>
+      <c r="E109" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F109" t="n">
+        <v>2025</v>
+      </c>
       <c r="G109" t="s">
         <v>224</v>
       </c>
@@ -3519,8 +3951,12 @@
       <c r="D110" t="s">
         <v>10</v>
       </c>
-      <c r="E110" s="1"/>
-      <c r="F110"/>
+      <c r="E110" s="1" t="n">
+        <v>45705</v>
+      </c>
+      <c r="F110" t="n">
+        <v>2025</v>
+      </c>
       <c r="G110" t="s">
         <v>226</v>
       </c>
@@ -3538,8 +3974,12 @@
       <c r="D111" t="s">
         <v>10</v>
       </c>
-      <c r="E111" s="1"/>
-      <c r="F111"/>
+      <c r="E111" s="1" t="n">
+        <v>45712</v>
+      </c>
+      <c r="F111" t="n">
+        <v>2025</v>
+      </c>
       <c r="G111" t="s">
         <v>228</v>
       </c>
@@ -3557,8 +3997,12 @@
       <c r="D112" t="s">
         <v>17</v>
       </c>
-      <c r="E112" s="1"/>
-      <c r="F112"/>
+      <c r="E112" s="1" t="n">
+        <v>45712</v>
+      </c>
+      <c r="F112" t="n">
+        <v>2025</v>
+      </c>
       <c r="G112" t="s">
         <v>232</v>
       </c>
@@ -3576,8 +4020,12 @@
       <c r="D113" t="s">
         <v>10</v>
       </c>
-      <c r="E113" s="1"/>
-      <c r="F113"/>
+      <c r="E113" s="1" t="n">
+        <v>45712</v>
+      </c>
+      <c r="F113" t="n">
+        <v>2025</v>
+      </c>
       <c r="G113" t="s">
         <v>234</v>
       </c>
@@ -3595,8 +4043,12 @@
       <c r="D114" t="s">
         <v>17</v>
       </c>
-      <c r="E114" s="1"/>
-      <c r="F114"/>
+      <c r="E114" s="1" t="n">
+        <v>45717</v>
+      </c>
+      <c r="F114" t="n">
+        <v>2025</v>
+      </c>
       <c r="G114"/>
     </row>
     <row r="115">
@@ -3612,8 +4064,12 @@
       <c r="D115" t="s">
         <v>17</v>
       </c>
-      <c r="E115" s="1"/>
-      <c r="F115"/>
+      <c r="E115" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="F115" t="n">
+        <v>2025</v>
+      </c>
       <c r="G115"/>
     </row>
     <row r="116">
@@ -3629,8 +4085,12 @@
       <c r="D116" t="s">
         <v>10</v>
       </c>
-      <c r="E116" s="1"/>
-      <c r="F116"/>
+      <c r="E116" s="1" t="n">
+        <v>45719</v>
+      </c>
+      <c r="F116" t="n">
+        <v>2025</v>
+      </c>
       <c r="G116" t="s">
         <v>238</v>
       </c>
@@ -3648,8 +4108,12 @@
       <c r="D117" t="s">
         <v>10</v>
       </c>
-      <c r="E117" s="1"/>
-      <c r="F117"/>
+      <c r="E117" s="1" t="n">
+        <v>45719</v>
+      </c>
+      <c r="F117" t="n">
+        <v>2025</v>
+      </c>
       <c r="G117" t="s">
         <v>240</v>
       </c>
@@ -3667,8 +4131,12 @@
       <c r="D118" t="s">
         <v>10</v>
       </c>
-      <c r="E118" s="1"/>
-      <c r="F118"/>
+      <c r="E118" s="1" t="n">
+        <v>45719</v>
+      </c>
+      <c r="F118" t="n">
+        <v>2025</v>
+      </c>
       <c r="G118" t="s">
         <v>242</v>
       </c>
@@ -3686,8 +4154,12 @@
       <c r="D119" t="s">
         <v>17</v>
       </c>
-      <c r="E119" s="1"/>
-      <c r="F119"/>
+      <c r="E119" s="1" t="n">
+        <v>45726</v>
+      </c>
+      <c r="F119" t="n">
+        <v>2025</v>
+      </c>
       <c r="G119" t="s">
         <v>244</v>
       </c>
@@ -3705,8 +4177,12 @@
       <c r="D120" t="s">
         <v>10</v>
       </c>
-      <c r="E120" s="1"/>
-      <c r="F120"/>
+      <c r="E120" s="1" t="n">
+        <v>45740</v>
+      </c>
+      <c r="F120" t="n">
+        <v>2025</v>
+      </c>
       <c r="G120" t="s">
         <v>246</v>
       </c>
@@ -3724,8 +4200,12 @@
       <c r="D121" t="s">
         <v>10</v>
       </c>
-      <c r="E121" s="1"/>
-      <c r="F121"/>
+      <c r="E121" s="1" t="n">
+        <v>45743</v>
+      </c>
+      <c r="F121" t="n">
+        <v>2025</v>
+      </c>
       <c r="G121" t="s">
         <v>248</v>
       </c>
@@ -3743,8 +4223,12 @@
       <c r="D122" t="s">
         <v>10</v>
       </c>
-      <c r="E122" s="1"/>
-      <c r="F122"/>
+      <c r="E122" s="1" t="n">
+        <v>45743</v>
+      </c>
+      <c r="F122" t="n">
+        <v>2025</v>
+      </c>
       <c r="G122" t="s">
         <v>250</v>
       </c>
@@ -3762,8 +4246,12 @@
       <c r="D123" t="s">
         <v>10</v>
       </c>
-      <c r="E123" s="1"/>
-      <c r="F123"/>
+      <c r="E123" s="1" t="n">
+        <v>45748</v>
+      </c>
+      <c r="F123" t="n">
+        <v>2025</v>
+      </c>
       <c r="G123" t="s">
         <v>252</v>
       </c>
@@ -3781,8 +4269,12 @@
       <c r="D124" t="s">
         <v>17</v>
       </c>
-      <c r="E124" s="1"/>
-      <c r="F124"/>
+      <c r="E124" s="1" t="n">
+        <v>45748</v>
+      </c>
+      <c r="F124" t="n">
+        <v>2025</v>
+      </c>
       <c r="G124" t="s">
         <v>254</v>
       </c>
@@ -3800,8 +4292,12 @@
       <c r="D125" t="s">
         <v>17</v>
       </c>
-      <c r="E125" s="1"/>
-      <c r="F125"/>
+      <c r="E125" s="1" t="n">
+        <v>45748</v>
+      </c>
+      <c r="F125" t="n">
+        <v>2025</v>
+      </c>
       <c r="G125"/>
     </row>
     <row r="126">
@@ -3817,8 +4313,12 @@
       <c r="D126" t="s">
         <v>10</v>
       </c>
-      <c r="E126" s="1"/>
-      <c r="F126"/>
+      <c r="E126" s="1" t="n">
+        <v>45754</v>
+      </c>
+      <c r="F126" t="n">
+        <v>2025</v>
+      </c>
       <c r="G126" t="s">
         <v>257</v>
       </c>
@@ -3836,8 +4336,12 @@
       <c r="D127" t="s">
         <v>10</v>
       </c>
-      <c r="E127" s="1"/>
-      <c r="F127"/>
+      <c r="E127" s="1" t="n">
+        <v>45784</v>
+      </c>
+      <c r="F127" t="n">
+        <v>2025</v>
+      </c>
       <c r="G127" t="s">
         <v>259</v>
       </c>
@@ -3855,8 +4359,12 @@
       <c r="D128" t="s">
         <v>17</v>
       </c>
-      <c r="E128" s="1"/>
-      <c r="F128"/>
+      <c r="E128" s="1" t="n">
+        <v>45796</v>
+      </c>
+      <c r="F128" t="n">
+        <v>2025</v>
+      </c>
       <c r="G128"/>
     </row>
     <row r="129">
@@ -3872,8 +4380,12 @@
       <c r="D129" t="s">
         <v>10</v>
       </c>
-      <c r="E129" s="1"/>
-      <c r="F129"/>
+      <c r="E129" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="F129" t="n">
+        <v>2025</v>
+      </c>
       <c r="G129" t="s">
         <v>262</v>
       </c>
@@ -3891,8 +4403,12 @@
       <c r="D130" t="s">
         <v>10</v>
       </c>
-      <c r="E130" s="1"/>
-      <c r="F130"/>
+      <c r="E130" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="F130" t="n">
+        <v>2025</v>
+      </c>
       <c r="G130" t="s">
         <v>264</v>
       </c>
@@ -3910,8 +4426,12 @@
       <c r="D131" t="s">
         <v>17</v>
       </c>
-      <c r="E131" s="1"/>
-      <c r="F131"/>
+      <c r="E131" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="F131" t="n">
+        <v>2025</v>
+      </c>
       <c r="G131"/>
     </row>
     <row r="132">
@@ -3927,8 +4447,12 @@
       <c r="D132" t="s">
         <v>17</v>
       </c>
-      <c r="E132" s="1"/>
-      <c r="F132"/>
+      <c r="E132" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="F132" t="n">
+        <v>2025</v>
+      </c>
       <c r="G132"/>
     </row>
     <row r="133">
@@ -3944,8 +4468,12 @@
       <c r="D133" t="s">
         <v>10</v>
       </c>
-      <c r="E133" s="1"/>
-      <c r="F133"/>
+      <c r="E133" s="1" t="n">
+        <v>45852</v>
+      </c>
+      <c r="F133" t="n">
+        <v>2025</v>
+      </c>
       <c r="G133" t="s">
         <v>268</v>
       </c>
@@ -3963,8 +4491,12 @@
       <c r="D134" t="s">
         <v>17</v>
       </c>
-      <c r="E134" s="1"/>
-      <c r="F134"/>
+      <c r="E134" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="F134" t="n">
+        <v>2025</v>
+      </c>
       <c r="G134"/>
     </row>
     <row r="135">
@@ -3980,8 +4512,12 @@
       <c r="D135" t="s">
         <v>10</v>
       </c>
-      <c r="E135" s="1"/>
-      <c r="F135"/>
+      <c r="E135" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F135" t="n">
+        <v>2025</v>
+      </c>
       <c r="G135" t="s">
         <v>271</v>
       </c>
@@ -3999,8 +4535,12 @@
       <c r="D136" t="s">
         <v>10</v>
       </c>
-      <c r="E136" s="1"/>
-      <c r="F136"/>
+      <c r="E136" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F136" t="n">
+        <v>2025</v>
+      </c>
       <c r="G136" t="s">
         <v>273</v>
       </c>
@@ -4018,8 +4558,12 @@
       <c r="D137" t="s">
         <v>10</v>
       </c>
-      <c r="E137" s="1"/>
-      <c r="F137"/>
+      <c r="E137" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F137" t="n">
+        <v>2025</v>
+      </c>
       <c r="G137" t="s">
         <v>275</v>
       </c>
@@ -4037,8 +4581,12 @@
       <c r="D138" t="s">
         <v>10</v>
       </c>
-      <c r="E138" s="1"/>
-      <c r="F138"/>
+      <c r="E138" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F138" t="n">
+        <v>2025</v>
+      </c>
       <c r="G138" t="s">
         <v>277</v>
       </c>
@@ -4056,8 +4604,12 @@
       <c r="D139" t="s">
         <v>10</v>
       </c>
-      <c r="E139" s="1"/>
-      <c r="F139"/>
+      <c r="E139" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F139" t="n">
+        <v>2025</v>
+      </c>
       <c r="G139" t="s">
         <v>279</v>
       </c>
@@ -4075,8 +4627,12 @@
       <c r="D140" t="s">
         <v>10</v>
       </c>
-      <c r="E140" s="1"/>
-      <c r="F140"/>
+      <c r="E140" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F140" t="n">
+        <v>2025</v>
+      </c>
       <c r="G140" t="s">
         <v>281</v>
       </c>
@@ -4094,8 +4650,12 @@
       <c r="D141" t="s">
         <v>10</v>
       </c>
-      <c r="E141" s="1"/>
-      <c r="F141"/>
+      <c r="E141" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F141" t="n">
+        <v>2025</v>
+      </c>
       <c r="G141" t="s">
         <v>283</v>
       </c>
@@ -4113,8 +4673,12 @@
       <c r="D142" t="s">
         <v>10</v>
       </c>
-      <c r="E142" s="1"/>
-      <c r="F142"/>
+      <c r="E142" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F142" t="n">
+        <v>2025</v>
+      </c>
       <c r="G142" t="s">
         <v>285</v>
       </c>
@@ -4132,8 +4696,12 @@
       <c r="D143" t="s">
         <v>10</v>
       </c>
-      <c r="E143" s="1"/>
-      <c r="F143"/>
+      <c r="E143" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F143" t="n">
+        <v>2025</v>
+      </c>
       <c r="G143" t="s">
         <v>287</v>
       </c>
@@ -4151,8 +4719,12 @@
       <c r="D144" t="s">
         <v>10</v>
       </c>
-      <c r="E144" s="1"/>
-      <c r="F144"/>
+      <c r="E144" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F144" t="n">
+        <v>2025</v>
+      </c>
       <c r="G144" t="s">
         <v>289</v>
       </c>
@@ -4170,8 +4742,12 @@
       <c r="D145" t="s">
         <v>10</v>
       </c>
-      <c r="E145" s="1"/>
-      <c r="F145"/>
+      <c r="E145" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F145" t="n">
+        <v>2025</v>
+      </c>
       <c r="G145" t="s">
         <v>291</v>
       </c>
@@ -4189,8 +4765,12 @@
       <c r="D146" t="s">
         <v>10</v>
       </c>
-      <c r="E146" s="1"/>
-      <c r="F146"/>
+      <c r="E146" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F146" t="n">
+        <v>2025</v>
+      </c>
       <c r="G146" t="s">
         <v>293</v>
       </c>
@@ -4208,8 +4788,12 @@
       <c r="D147" t="s">
         <v>10</v>
       </c>
-      <c r="E147" s="1"/>
-      <c r="F147"/>
+      <c r="E147" s="1" t="n">
+        <v>45922</v>
+      </c>
+      <c r="F147" t="n">
+        <v>2025</v>
+      </c>
       <c r="G147" t="s">
         <v>295</v>
       </c>
@@ -4227,8 +4811,12 @@
       <c r="D148" t="s">
         <v>10</v>
       </c>
-      <c r="E148" s="1"/>
-      <c r="F148"/>
+      <c r="E148" s="1" t="n">
+        <v>45929</v>
+      </c>
+      <c r="F148" t="n">
+        <v>2025</v>
+      </c>
       <c r="G148" t="s">
         <v>297</v>
       </c>
@@ -4246,8 +4834,12 @@
       <c r="D149" t="s">
         <v>10</v>
       </c>
-      <c r="E149" s="1"/>
-      <c r="F149"/>
+      <c r="E149" s="1" t="n">
+        <v>45929</v>
+      </c>
+      <c r="F149" t="n">
+        <v>2025</v>
+      </c>
       <c r="G149" t="s">
         <v>299</v>
       </c>
@@ -4265,8 +4857,12 @@
       <c r="D150" t="s">
         <v>10</v>
       </c>
-      <c r="E150" s="1"/>
-      <c r="F150"/>
+      <c r="E150" s="1" t="n">
+        <v>45931</v>
+      </c>
+      <c r="F150" t="n">
+        <v>2025</v>
+      </c>
       <c r="G150" t="s">
         <v>301</v>
       </c>
@@ -4284,8 +4880,12 @@
       <c r="D151" t="s">
         <v>10</v>
       </c>
-      <c r="E151" s="1"/>
-      <c r="F151"/>
+      <c r="E151" s="1" t="n">
+        <v>45939</v>
+      </c>
+      <c r="F151" t="n">
+        <v>2025</v>
+      </c>
       <c r="G151" t="s">
         <v>303</v>
       </c>
@@ -4303,8 +4903,12 @@
       <c r="D152" t="s">
         <v>10</v>
       </c>
-      <c r="E152" s="1"/>
-      <c r="F152"/>
+      <c r="E152" s="1" t="n">
+        <v>45944</v>
+      </c>
+      <c r="F152" t="n">
+        <v>2025</v>
+      </c>
       <c r="G152" t="s">
         <v>277</v>
       </c>
@@ -4322,8 +4926,12 @@
       <c r="D153" t="s">
         <v>10</v>
       </c>
-      <c r="E153" s="1"/>
-      <c r="F153"/>
+      <c r="E153" s="1" t="n">
+        <v>45951</v>
+      </c>
+      <c r="F153" t="n">
+        <v>2025</v>
+      </c>
       <c r="G153" t="s">
         <v>306</v>
       </c>
@@ -4341,8 +4949,12 @@
       <c r="D154" t="s">
         <v>10</v>
       </c>
-      <c r="E154" s="1"/>
-      <c r="F154"/>
+      <c r="E154" s="1" t="n">
+        <v>45962</v>
+      </c>
+      <c r="F154" t="n">
+        <v>2025</v>
+      </c>
       <c r="G154" t="s">
         <v>308</v>
       </c>
@@ -4360,8 +4972,12 @@
       <c r="D155" t="s">
         <v>10</v>
       </c>
-      <c r="E155" s="1"/>
-      <c r="F155"/>
+      <c r="E155" s="1" t="n">
+        <v>45976</v>
+      </c>
+      <c r="F155" t="n">
+        <v>2025</v>
+      </c>
       <c r="G155" t="s">
         <v>310</v>
       </c>
@@ -4379,8 +4995,12 @@
       <c r="D156" t="s">
         <v>10</v>
       </c>
-      <c r="E156" s="1"/>
-      <c r="F156"/>
+      <c r="E156" s="1" t="n">
+        <v>46032</v>
+      </c>
+      <c r="F156" t="n">
+        <v>2026</v>
+      </c>
       <c r="G156" t="s">
         <v>312</v>
       </c>
@@ -4398,8 +5018,12 @@
       <c r="D157" t="s">
         <v>10</v>
       </c>
-      <c r="E157" s="1"/>
-      <c r="F157"/>
+      <c r="E157" s="1" t="n">
+        <v>46065</v>
+      </c>
+      <c r="F157" t="n">
+        <v>2026</v>
+      </c>
       <c r="G157" t="s">
         <v>314</v>
       </c>
@@ -4440,8 +5064,12 @@
       <c r="D159" t="s">
         <v>10</v>
       </c>
-      <c r="E159" s="1"/>
-      <c r="F159"/>
+      <c r="E159" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="F159" t="n">
+        <v>2026</v>
+      </c>
       <c r="G159" t="s">
         <v>318</v>
       </c>
@@ -4459,8 +5087,12 @@
       <c r="D160" t="s">
         <v>17</v>
       </c>
-      <c r="E160" s="1"/>
-      <c r="F160"/>
+      <c r="E160" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="F160" t="n">
+        <v>2026</v>
+      </c>
       <c r="G160"/>
     </row>
     <row r="161">
@@ -4476,8 +5108,12 @@
       <c r="D161" t="s">
         <v>10</v>
       </c>
-      <c r="E161" s="1"/>
-      <c r="F161"/>
+      <c r="E161" s="1" t="n">
+        <v>46079</v>
+      </c>
+      <c r="F161" t="n">
+        <v>2026</v>
+      </c>
       <c r="G161" t="s">
         <v>321</v>
       </c>
@@ -4495,8 +5131,12 @@
       <c r="D162" t="s">
         <v>10</v>
       </c>
-      <c r="E162" s="1"/>
-      <c r="F162"/>
+      <c r="E162" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="F162" t="n">
+        <v>2026</v>
+      </c>
       <c r="G162" t="s">
         <v>323</v>
       </c>
@@ -4514,8 +5154,12 @@
       <c r="D163" t="s">
         <v>10</v>
       </c>
-      <c r="E163" s="1"/>
-      <c r="F163"/>
+      <c r="E163" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="F163" t="n">
+        <v>2026</v>
+      </c>
       <c r="G163" t="s">
         <v>325</v>
       </c>
@@ -4533,8 +5177,12 @@
       <c r="D164" t="s">
         <v>10</v>
       </c>
-      <c r="E164" s="1"/>
-      <c r="F164"/>
+      <c r="E164" s="1" t="n">
+        <v>46083</v>
+      </c>
+      <c r="F164" t="n">
+        <v>2026</v>
+      </c>
       <c r="G164" t="s">
         <v>327</v>
       </c>
@@ -4552,8 +5200,12 @@
       <c r="D165" t="s">
         <v>10</v>
       </c>
-      <c r="E165" s="1"/>
-      <c r="F165"/>
+      <c r="E165" s="1" t="n">
+        <v>46083</v>
+      </c>
+      <c r="F165" t="n">
+        <v>2026</v>
+      </c>
       <c r="G165" t="s">
         <v>329</v>
       </c>
@@ -4571,8 +5223,12 @@
       <c r="D166" t="s">
         <v>10</v>
       </c>
-      <c r="E166" s="1"/>
-      <c r="F166"/>
+      <c r="E166" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="F166" t="n">
+        <v>2026</v>
+      </c>
       <c r="G166" t="s">
         <v>331</v>
       </c>
@@ -4590,8 +5246,12 @@
       <c r="D167" t="s">
         <v>10</v>
       </c>
-      <c r="E167" s="1"/>
-      <c r="F167"/>
+      <c r="E167" s="1" t="n">
+        <v>46069</v>
+      </c>
+      <c r="F167" t="n">
+        <v>2026</v>
+      </c>
       <c r="G167" t="s">
         <v>333</v>
       </c>
@@ -4609,8 +5269,12 @@
       <c r="D168" t="s">
         <v>10</v>
       </c>
-      <c r="E168" s="1"/>
-      <c r="F168"/>
+      <c r="E168" s="1" t="n">
+        <v>46070</v>
+      </c>
+      <c r="F168" t="n">
+        <v>2026</v>
+      </c>
       <c r="G168" t="s">
         <v>335</v>
       </c>
@@ -4628,8 +5292,12 @@
       <c r="D169" t="s">
         <v>10</v>
       </c>
-      <c r="E169" s="1"/>
-      <c r="F169"/>
+      <c r="E169" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="F169" t="n">
+        <v>2026</v>
+      </c>
       <c r="G169" t="s">
         <v>337</v>
       </c>
@@ -4647,8 +5315,12 @@
       <c r="D170" t="s">
         <v>10</v>
       </c>
-      <c r="E170" s="1"/>
-      <c r="F170"/>
+      <c r="E170" s="1" t="n">
+        <v>46090</v>
+      </c>
+      <c r="F170" t="n">
+        <v>2026</v>
+      </c>
       <c r="G170" t="s">
         <v>339</v>
       </c>
@@ -4666,8 +5338,12 @@
       <c r="D171" t="s">
         <v>10</v>
       </c>
-      <c r="E171" s="1"/>
-      <c r="F171"/>
+      <c r="E171" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="F171" t="n">
+        <v>2026</v>
+      </c>
       <c r="G171" t="s">
         <v>341</v>
       </c>
@@ -4685,8 +5361,12 @@
       <c r="D172" t="s">
         <v>10</v>
       </c>
-      <c r="E172" s="1"/>
-      <c r="F172"/>
+      <c r="E172" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="F172" t="n">
+        <v>2026</v>
+      </c>
       <c r="G172" t="s">
         <v>343</v>
       </c>
@@ -4704,8 +5384,12 @@
       <c r="D173" t="s">
         <v>10</v>
       </c>
-      <c r="E173" s="1"/>
-      <c r="F173"/>
+      <c r="E173" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="F173" t="n">
+        <v>2026</v>
+      </c>
       <c r="G173"/>
     </row>
     <row r="174">
@@ -4721,8 +5405,12 @@
       <c r="D174" t="s">
         <v>10</v>
       </c>
-      <c r="E174" s="1"/>
-      <c r="F174"/>
+      <c r="E174" s="1" t="n">
+        <v>46083</v>
+      </c>
+      <c r="F174" t="n">
+        <v>2026</v>
+      </c>
       <c r="G174" t="s">
         <v>346</v>
       </c>
@@ -4740,8 +5428,12 @@
       <c r="D175" t="s">
         <v>10</v>
       </c>
-      <c r="E175" s="1"/>
-      <c r="F175"/>
+      <c r="E175" s="1" t="n">
+        <v>46097</v>
+      </c>
+      <c r="F175" t="n">
+        <v>2026</v>
+      </c>
       <c r="G175" t="s">
         <v>348</v>
       </c>
@@ -4759,8 +5451,12 @@
       <c r="D176" t="s">
         <v>10</v>
       </c>
-      <c r="E176" s="1"/>
-      <c r="F176"/>
+      <c r="E176" s="1" t="n">
+        <v>46125</v>
+      </c>
+      <c r="F176" t="n">
+        <v>2026</v>
+      </c>
       <c r="G176" t="s">
         <v>350</v>
       </c>
@@ -4778,8 +5474,12 @@
       <c r="D177" t="s">
         <v>10</v>
       </c>
-      <c r="E177" s="1"/>
-      <c r="F177"/>
+      <c r="E177" s="1" t="n">
+        <v>46126</v>
+      </c>
+      <c r="F177" t="n">
+        <v>2026</v>
+      </c>
       <c r="G177" t="s">
         <v>352</v>
       </c>
@@ -4797,8 +5497,12 @@
       <c r="D178" t="s">
         <v>17</v>
       </c>
-      <c r="E178" s="1"/>
-      <c r="F178"/>
+      <c r="E178" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="F178" t="n">
+        <v>2026</v>
+      </c>
       <c r="G178"/>
     </row>
     <row r="179">
@@ -4814,8 +5518,12 @@
       <c r="D179" t="s">
         <v>17</v>
       </c>
-      <c r="E179" s="1"/>
-      <c r="F179"/>
+      <c r="E179" s="1" t="n">
+        <v>46082</v>
+      </c>
+      <c r="F179" t="n">
+        <v>2026</v>
+      </c>
       <c r="G179"/>
     </row>
     <row r="180">
@@ -4831,8 +5539,12 @@
       <c r="D180" t="s">
         <v>17</v>
       </c>
-      <c r="E180" s="1"/>
-      <c r="F180"/>
+      <c r="E180" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="F180" t="n">
+        <v>2026</v>
+      </c>
       <c r="G180"/>
     </row>
     <row r="181">
@@ -4848,8 +5560,12 @@
       <c r="D181" t="s">
         <v>17</v>
       </c>
-      <c r="E181" s="1"/>
-      <c r="F181"/>
+      <c r="E181" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="F181" t="n">
+        <v>2026</v>
+      </c>
       <c r="G181"/>
     </row>
     <row r="182">
@@ -4865,8 +5581,12 @@
       <c r="D182" t="s">
         <v>10</v>
       </c>
-      <c r="E182" s="1"/>
-      <c r="F182"/>
+      <c r="E182" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="F182" t="n">
+        <v>2026</v>
+      </c>
       <c r="G182" t="s">
         <v>358</v>
       </c>
@@ -4884,8 +5604,12 @@
       <c r="D183" t="s">
         <v>10</v>
       </c>
-      <c r="E183" s="1"/>
-      <c r="F183"/>
+      <c r="E183" s="1" t="n">
+        <v>46155</v>
+      </c>
+      <c r="F183" t="n">
+        <v>2026</v>
+      </c>
       <c r="G183" t="s">
         <v>360</v>
       </c>
@@ -4903,8 +5627,12 @@
       <c r="D184" t="s">
         <v>10</v>
       </c>
-      <c r="E184" s="1"/>
-      <c r="F184"/>
+      <c r="E184" s="1" t="n">
+        <v>46160</v>
+      </c>
+      <c r="F184" t="n">
+        <v>2026</v>
+      </c>
       <c r="G184" t="s">
         <v>362</v>
       </c>
@@ -4922,8 +5650,12 @@
       <c r="D185" t="s">
         <v>10</v>
       </c>
-      <c r="E185" s="1"/>
-      <c r="F185"/>
+      <c r="E185" s="1" t="n">
+        <v>46277</v>
+      </c>
+      <c r="F185" t="n">
+        <v>2026</v>
+      </c>
       <c r="G185" t="s">
         <v>364</v>
       </c>
@@ -4941,8 +5673,12 @@
       <c r="D186" t="s">
         <v>10</v>
       </c>
-      <c r="E186" s="1"/>
-      <c r="F186"/>
+      <c r="E186" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="F186" t="n">
+        <v>2026</v>
+      </c>
       <c r="G186" t="s">
         <v>366</v>
       </c>
@@ -4960,8 +5696,12 @@
       <c r="D187" t="s">
         <v>17</v>
       </c>
-      <c r="E187" s="1"/>
-      <c r="F187"/>
+      <c r="E187" s="1" t="n">
+        <v>46113</v>
+      </c>
+      <c r="F187" t="n">
+        <v>2026</v>
+      </c>
       <c r="G187"/>
     </row>
   </sheetData>

</xml_diff>